<commit_message>
fix(caisse-ml): mapping en-têtes tolérant (suffixe * du modèle) + fixture fidèle modèle + tests (4.2)
Le modèle téléchargé (buildModeleWorkbook) annote les colonnes requises avec
un suffixe « * » (Client *, Date encaissement *, Montant (DH) *, Référence *),
mais le parseur lisait les cellules via row[header] EXACT sans « * » → toutes
les lignes rejetées « client_absent » sur un fichier conforme au modèle.

- cell() : chemin rapide exact puis fallback tolérant via normHeader() qui
  ignore le/les « * » final(aux), la casse, le trim et les espaces multiples.
- Fixture régénérée FIDÈLE AU MODÈLE (en-têtes annotés « * ») : 10 lignes
  → 2 OK / 7 rejets (un par motif) / 1 doublon intra-fichier.
- Tests anti-régression : en-têtes « * », variantes casse/espaces, et client
  actif dont le nom est aussi dans archivedNames → accepté (réserve QA 4.2),
  + smoke fixture confirmant 10/2/7/1.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/canevas_encaissements_demo.xlsx
+++ b/tests/fixtures/canevas_encaissements_demo.xlsx
@@ -401,19 +401,19 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Client</v>
+        <v>Client *</v>
       </c>
       <c r="B1" t="str">
-        <v>Date encaissement</v>
+        <v>Date encaissement *</v>
       </c>
       <c r="C1" t="str">
-        <v>Montant (DH)</v>
+        <v>Montant (DH) *</v>
       </c>
       <c r="D1" t="str">
         <v>Mode</v>
       </c>
       <c r="E1" t="str">
-        <v>Référence</v>
+        <v>Référence *</v>
       </c>
       <c r="F1" t="str">
         <v>Motif</v>

</xml_diff>